<commit_message>
chore: auto sync from private repo
</commit_message>
<xml_diff>
--- a/assets/dungeon_paths.xlsx
+++ b/assets/dungeon_paths.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="副本路径配置" sheetId="1" r:id="R3a61702fc4064726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="难度映射" sheetId="2" r:id="Rf694b006e61f4017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="副本路径配置" sheetId="1" r:id="R52c84897bf0b4c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="难度映射" sheetId="2" r:id="Ra9736f947a8c4182"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -456,7 +456,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C3" s="11" t="str">
-        <x:v>[[-681.182,580],[-362.894,580],[-285.287,584.312],[-220.614,583.45],[-220.614,583.45],[-148.181,577.414],[-70.574,570.515],[9.62,556.718],[84.64,550.682],[157.073,536.885],[219.159,525.675],[278.658,496.357],[330.396,454.104],[361.439,391.156],[356.265,323.034],[312.288,260.086],[260.55,212.659],[182.943,175.58],[110.51,195.413],[61.359,254.049],[51.011,317.859],[51.011,372.184],[87.227,434.27],[162.247,442.03],[232.093,412.712],[250.201,362.699],[201.05,299.751],[157.073,257.498],[102.748,223.006],[35.489,180.753],[-62.813,161.782],[-158.528,158.333],[-230.961,180.753],[-305.981,229.042],[-334.437,303.2],[-331.85,382.532],[-282.699,435.995],[-223.2,468.762],[-143.006,480.834],[-67.986,467.037],[-42.117,393.741],[-42.117,325.619],[-75.747,274.744],[-135.246,232.491],[-197.332,182.478],[-241.309,129.878],[-285.286,66.93],[-321.503,-1.192],[-342.198,-74.488],[-313.742,-145.197],[-256.83,-213.319],[-174.049,-229.703],[-106.79,-204.696],[-67.986,-158.994],[-34.356,-105.531],[-29.182,-36.547],[-67.986,23.814],[-117.137,50.546],[-174.049,50.546],[-220.613,0.533],[-228.374,-62.415],[-186.984,-107.255],[-135.246,-159.855],[-67.987,-196.934],[1.859,-223.665],[87.227,-232.288],[149.312,-239.187],[219.159,-234.875],[276.071,-212.455],[314.875,-161.579],[335.57,-95.182],[332.983,-33.959],[314.875,22.091],[268.311,57.445],[198.465,79.865],[126.032,66.068],[87.228,3.12],[87.228,-59.828],[128.618,-109.841],[190.704,-167.615],[252.79,-235.737],[284.684,-286.055],[257.554,-330],[-286.029,-330],[-323.4,-380],[-287.727,-430],[308.515,-430],[340.79,-480],[310.214,-530],[97.877,-516.977],[72.397,-536.229],[48.615,-593.418]]</x:v>
+        <x:v>[[0,580],[318.288,580],[395.895,584.312],[460.568,583.45],[460.568,583.45],[533.001,577.414],[610.608,570.515],[690.802,556.718],[765.822,550.682],[838.255,536.885],[900.341,525.675],[959.84,496.357],[1011.578,454.104],[1042.621,391.156],[1037.447,323.034],[993.47,260.086],[941.732,212.659],[864.125,175.58],[791.692,195.413],[742.541,254.049],[732.193,317.859],[732.193,372.184],[768.409,434.27],[843.429,442.03],[913.275,412.712],[931.383,362.699],[882.232,299.751],[838.255,257.498],[783.93,223.006],[716.671,180.753],[618.369,161.782],[522.654,158.333],[450.221,180.753],[375.201,229.042],[346.745,303.2],[349.332,382.532],[398.483,435.995],[457.982,468.762],[538.176,480.834],[613.196,467.037],[639.065,393.741],[639.065,325.619],[605.435,274.744],[545.936,232.491],[483.85,182.478],[439.873,129.878],[395.896,66.93],[359.679,-1.192],[338.984,-74.488],[367.44,-145.197],[424.352,-213.319],[507.133,-229.703],[574.392,-204.696],[613.196,-158.994],[646.826,-105.531],[652,-36.547],[613.196,23.814],[564.045,50.546],[507.133,50.546],[460.569,0.533],[452.808,-62.415],[494.198,-107.255],[545.936,-159.855],[613.195,-196.934],[683.041,-223.665],[768.409,-232.288],[830.494,-239.187],[900.341,-234.875],[957.253,-212.455],[996.057,-161.579],[1016.752,-95.182],[1014.165,-33.959],[996.057,22.091],[949.493,57.445],[879.647,79.865],[807.214,66.068],[768.41,3.12],[768.41,-59.828],[809.8,-109.841],[871.886,-167.615],[933.972,-235.737],[965.866,-286.055],[938.736,-330],[395.153,-330],[357.782,-380],[393.455,-430],[989.697,-430],[1021.972,-480],[991.396,-530],[779.059,-516.977],[753.579,-536.229],[729.797,-593.418]]</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -467,7 +467,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>[[-700,630],[-356.479,630],[-318.872,605.373],[-300,570],[-300,200],[-250,150],[-200,200],[-200,580],[-150,630],[-100,580],[-100,200],[-50,150],[0,200],[0,580],[50,630],[100,580],[100,580],[100,200],[150,150],[200,200],[200,580],[250,630],[300,580],[300,150],[261.625,100.881],[191.016,50],[-213.452,50],[-294.806,27.743],[-330,-36.726],[-330,-400],[-312.348,-426.862],[-268,-450],[268,-450],[301.769,-433.115],[330,-400],[330,-110.656],[303.138,-69.212],[268,-50],[-161.027,-50],[-196.332,-65.35],[-230,-91.445],[-230,-300.203],[-215.418,-330.903],[-180.113,-350],[195.958,-350],[219.75,-332.348],[238.937,-297.539],[238.937,-219.254],[199.795,-163.228],[164.491,-150],[-111.038,-150],[-141.738,-163.048],[-157.088,-200.655],[-124.086,-250],[-64.99,-257.675],[0,-273.792],[30.7,-316.004],[56.795,-362.821],[29.933,-423.453],[-8.442,-465.665],[-9.977,-512.482],[11.001,-560.947]]</x:v>
+        <x:v>[[0,630],[343.521,630],[381.128,605.373],[400,570],[400,200],[450,150],[500,200],[500,580],[550,630],[600,580],[600,200],[650,150],[700,200],[700,580],[750,630],[800,580],[800,580],[800,200],[850,150],[900,200],[900,580],[950,630],[1000,580],[1000,150],[961.625,100.881],[891.016,50],[486.548,50],[405.194,27.743],[370,-36.726],[370,-400],[387.652,-426.862],[432,-450],[968,-450],[1001.769,-433.115],[1030,-400],[1030,-110.656],[1003.138,-69.212],[968,-50],[538.973,-50],[503.668,-65.35],[470,-91.445],[470,-300.203],[484.582,-330.903],[519.887,-350],[895.958,-350],[919.75,-332.348],[938.937,-297.539],[938.937,-219.254],[899.795,-163.228],[864.491,-150],[588.962,-150],[558.262,-163.048],[542.912,-200.655],[575.914,-250],[635.01,-257.675],[700,-273.792],[730.7,-316.004],[756.795,-362.821],[729.933,-423.453],[691.558,-465.665],[690.023,-512.482],[711.001,-560.947]]</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
@@ -478,7 +478,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>[[-645.448,1100],[-366.001,631.782],[-222.568,700.201],[-49.46,736.238],[111.677,731.373],[276.983,692.325],[418.872,621.744],[527.683,536.838],[634.021,419.784],[708.21,282.121],[745.305,155.175],[755.197,13.391],[740.359,-146.528],[695.845,-284.19],[616.71,-402.893],[515.318,-531.488],[384.25,-618.867],[230.925,-676.57],[85.019,-697.178],[-75.725,-683.164],[-229.05,-634.529],[-370.01,-543.853],[-476.348,-435.866],[-550.537,-317.987],[-595.051,-187.743],[-622.254,-48.431],[-604.943,85.11],[-557.956,254.921],[-468.929,382.692],[-352.699,500.571],[-226.577,564.044],[-88.09,605.26],[70.181,609.382],[203.722,581.355],[334.79,530.247],[455.966,430.503],[547.466,330.759],[614.236,184.853],[629.074,35.65],[621.655,-111.08],[579.614,-242.972],[512.843,-342.716],[411.451,-442.46],[300.167,-522.42],[156.734,-566.109],[-6.483,-578.474],[-174.646,-524.893],[-295.822,-446.582],[-387.322,-355.906],[-456.566,-245.446],[-491.188,-100.364],[-493.661,27.407],[-461.512,157.651],[-399.687,282.949],[-290.876,395.882],[-137.551,474.193],[38.031,498.099],[218.559,460.18],[342.208,375.274],[446.073,275.53],[498.006,151.057],[515.317,-10.511],[478.222,-167.133],[386.722,-316.336],[248.235,-418.553],[62.761,-458.945],[-147.443,-405.364],[-278.511,-299.85],[-360.119,-174.552],[-382.376,-4.741],[-340.335,147.76],[-253.781,260.693],[-140.024,339.004],[13.301,374.45],[166.626,347.247],[295.221,262.341],[371.883,152.705],[391.667,18.34],[369.41,-118.498],[285.329,-242.971],[149.315,-322.931],[-38.632,-328.701],[-159.808,-253.688],[-243.889,-140.755],[-261.2,-13.808],[-229.051,111.49],[-140.024,206.288],[-8.956,259.869],[129.531,236.788],[228.45,156.828],[272.964,49.665],[253.18,-79.754],[161.68,-192.687],[5.882,-210.822],[-112.821,-122.619],[-137.551,-2.267],[-85.618,102.423],[20.72,142.815],[122.112,100.773],[146.842,48.016],[141.896,-32.768],[97.382,-105.309],[35.557,-50.079]]</x:v>
+        <x:v>[[0,1100],[279.447,631.782],[422.88,700.201],[595.988,736.238],[757.125,731.373],[922.431,692.325],[1064.32,621.744],[1173.131,536.838],[1279.469,419.784],[1353.658,282.121],[1390.753,155.175],[1400.645,13.391],[1385.807,-146.528],[1341.293,-284.19],[1262.158,-402.893],[1160.766,-531.488],[1029.698,-618.867],[876.373,-676.57],[730.467,-697.178],[569.723,-683.164],[416.398,-634.529],[275.438,-543.853],[169.1,-435.866],[94.911,-317.987],[50.397,-187.743],[23.194,-48.431],[40.505,85.11],[87.492,254.921],[176.519,382.692],[292.749,500.571],[418.871,564.044],[557.358,605.26],[715.629,609.382],[849.17,581.355],[980.238,530.247],[1101.414,430.503],[1192.914,330.759],[1259.684,184.853],[1274.522,35.65],[1267.103,-111.08],[1225.062,-242.972],[1158.291,-342.716],[1056.899,-442.46],[945.615,-522.42],[802.182,-566.109],[638.965,-578.474],[470.802,-524.893],[349.626,-446.582],[258.126,-355.906],[188.882,-245.446],[154.26,-100.364],[151.787,27.407],[183.936,157.651],[245.761,282.949],[354.572,395.882],[507.897,474.193],[683.479,498.099],[864.007,460.18],[987.656,375.274],[1091.521,275.53],[1143.454,151.057],[1160.765,-10.511],[1123.67,-167.133],[1032.17,-316.336],[893.683,-418.553],[708.209,-458.945],[498.005,-405.364],[366.937,-299.85],[285.329,-174.552],[263.072,-4.741],[305.113,147.76],[391.667,260.693],[505.424,339.004],[658.749,374.45],[812.074,347.247],[940.669,262.341],[1017.331,152.705],[1037.115,18.34],[1014.858,-118.498],[930.777,-242.971],[794.763,-322.931],[606.816,-328.701],[485.64,-253.688],[401.559,-140.755],[384.248,-13.808],[416.397,111.49],[505.424,206.288],[636.492,259.869],[774.979,236.788],[873.898,156.828],[918.412,49.665],[898.628,-79.754],[807.128,-192.687],[651.33,-210.822],[532.627,-122.619],[507.897,-2.267],[559.83,102.423],[666.168,142.815],[767.56,100.773],[792.29,48.016],[787.344,-32.768],[742.83,-105.309],[681.005,-50.079]]</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
@@ -489,7 +489,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>[[-550,50],[-474.625,135.027],[-369.561,202.123],[-200,260],[-264.226,309.631],[-328.828,351.777],[-365.984,408.893],[-400.103,480.709],[-385.132,558.057],[-321.613,583.332],[-253.975,543.41],[-190,500],[-136.164,547.859],[-76.012,594.994],[0,630],[79.496,596.678],[134.659,541.515],[190,500],[237.677,544.641],[280.364,559.341],[338.022,526.634],[373.224,468.976],[354.076,401.068],[319.144,340.914],[262.028,293.237],[207.677,260],[-200,260],[-550,260],[-550,-450],[-474.625,-364.97300000000007],[-369.561,-297.87700000000007],[-200,-240],[-264.226,-190.36900000000003],[-328.828,-148.22300000000007],[-365.984,-91.10700000000008],[-400.103,-19.291000000000054],[-385.132,58.0569999999999],[-321.613,83.332],[-253.975,43.40999999999997],[-190,1.1368683772161603e-13],[-136.164,47.85900000000004],[-76.012,94.99400000000003],[0,130.0000000000001],[79.49599999999998,96.678],[134.659,41.514999999999986],[190,1.1368683772161603e-13],[237.67700000000002,44.64099999999996],[280.36400000000003,59.34100000000001],[338.02199999999993,26.63400000000013],[373.22399999999993,-31.024],[354.076,-98.93200000000013],[319.144,-159.086],[262.028,-206.76300000000003],[207.67700000000002,-240],[-200,-240],[-550,-240],[-454.916,-282.687],[-369.812,-342.84],[-309.659,-400.498],[-249.506,-440.69],[-186.858,-396.049],[-129.2,-368.874],[-54.077,-356.669],[8.571,-354.445],[76.479,-362.472],[151.602,-380.208],[211.755,-402.935],[266.918,-445.622],[332.061,-418.447],[379.738,-376.301],[437.396,-339.145],[500,-284.794],[500,-97.933],[0,-97.933],[0,-205.493],[0,-308.062],[0,-430.592],[0,-530.666],[0,-588.324]]</x:v>
+        <x:v>[[0,50],[75.375,135.027],[180.439,202.123],[350,260],[285.774,309.631],[221.172,351.777],[184.016,408.893],[149.897,480.709],[164.868,558.057],[228.387,583.332],[296.025,543.41],[360,500],[413.836,547.859],[473.988,594.994],[550,630],[629.496,596.678],[684.659,541.515],[740,500],[787.677,544.641],[830.364,559.341],[888.022,526.634],[923.224,468.976],[904.076,401.068],[869.144,340.914],[812.028,293.237],[757.677,260],[350,260],[0,260],[0,-450],[75.375,-364.97300000000007],[180.439,-297.87700000000007],[350,-240],[285.774,-190.36900000000003],[221.172,-148.22300000000007],[184.016,-91.10700000000008],[149.897,-19.291000000000054],[164.868,58.0569999999999],[228.387,83.332],[296.025,43.40999999999997],[360,1.1368683772161603e-13],[413.836,47.85900000000004],[473.988,94.99400000000003],[550,130.0000000000001],[629.496,96.678],[684.659,41.514999999999986],[740,1.1368683772161603e-13],[787.677,44.64099999999996],[830.364,59.34100000000001],[888.022,26.63400000000013],[923.224,-31.024],[904.076,-98.93200000000013],[869.144,-159.086],[812.028,-206.76300000000003],[757.677,-240],[350,-240],[0,-240],[95.084,-282.687],[180.188,-342.84],[240.341,-400.498],[300.494,-440.69],[363.142,-396.049],[420.8,-368.874],[495.923,-356.669],[558.571,-354.445],[626.479,-362.472],[701.602,-380.208],[761.755,-402.935],[816.918,-445.622],[882.061,-418.447],[929.738,-376.301],[987.396,-339.145],[1050,-284.794],[1050,-97.933],[550,-97.933],[550,-205.493],[550,-308.062],[550,-430.592],[550,-530.666],[550,-588.324]]</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -500,7 +500,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>[[-620,480],[-444.643,480],[0,480],[-165,630],[-330,480],[-165,330],[0,480],[165,630],[330,480],[165,330],[0,480],[330,480],[330,180],[165,330],[0,180],[165,30],[330,180],[0,180],[-165,30],[-330,180],[-165,330],[0,180],[-330,180],[-330,-120],[-165,30],[0,-120],[-165,-270],[-330,-120],[0,-120],[165,-270],[330,-120],[165,30],[0,-120],[330,-120],[330,-420],[165,-270],[0,-420],[-165,-270],[-330,-420],[501.118,-420],[501.118,-270],[0,-270],[0,-335.158],[0,-420.281],[0,-507.9],[0,-583.041]]</x:v>
+        <x:v>[[0,480],[175.357,480],[620,480],[455,630],[290,480],[455,330],[620,480],[785,630],[950,480],[785,330],[620,480],[950,480],[950,180],[785,330],[620,180],[785,30],[950,180],[620,180],[455,30],[290,180],[455,330],[620,180],[290,180],[290,-120],[455,30],[620,-120],[455,-270],[290,-120],[620,-120],[785,-270],[950,-120],[785,30],[620,-120],[950,-120],[950,-420],[785,-270],[620,-420],[455,-270],[290,-420],[1121.118,-420],[1121.118,-270],[620,-270],[620,-335.158],[620,-420.281],[620,-507.9],[620,-583.041]]</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
@@ -511,7 +511,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>[[-600,530.0000000000001],[-100.00000000000006,530.0000000000001],[-67.86500000000001,552.6470000000003],[-40,590.0000000000001],[-64.78800000000001,631.0790000000001],[-100.00000000000006,650.0000000000001],[-143.216,632.1230000000002],[-160.00000000000003,590.0000000000001],[-144.41600000000003,557.3260000000004],[-100.00000000000006,530.0000000000001],[100,530.0000000000001],[134.07999999999998,552.919],[160,590.0000000000001],[136.10799999999995,632.245],[100,650.0000000000001],[61.25999999999999,634.7360000000002],[39.99999999999994,590.0000000000001],[52.60899999999998,552.8000000000001],[100,530.0000000000001],[500.00000000000006,530.0000000000001],[500.00000000000006,280.0000000000001],[0,280.0000000000001],[65.74199999999996,299.37700000000007],[115.12700000000001,329.43600000000004],[155.73799999999994,385.0190000000001],[160,450.0000000000001],[102.24599999999998,407.4230000000001],[50.714999999999975,390.24700000000007],[0,380],[-75.33200000000002,385.9760000000001],[-122.66100000000003,413.65700000000015],[-160.00000000000003,450.0000000000001],[-149.472,376.32500000000005],[-104.565,324.3280000000001],[-55.18000000000001,289.97300000000007],[0,280.0000000000001],[-500.0000000000001,280.0000000000001],[-500.0000000000001,30.000000000000114],[-100.00000000000006,30.000000000000114],[-67.86500000000001,52.647000000000276],[-40,90.00000000000011],[-64.78800000000001,131.07900000000006],[-100.00000000000006,150.0000000000001],[-143.216,132.12299999999993],[-160.00000000000009,90.00000000000011],[-144.41600000000008,57.326000000000136],[-100.00000000000006,30.000000000000114],[100,30.000000000000114],[134.07999999999998,52.919000000000096],[160,90.00000000000011],[136.10799999999995,132.24500000000012],[100,150.0000000000001],[61.25999999999999,134.7360000000001],[39.99999999999994,90.00000000000011],[52.608999999999924,52.800000000000296],[100,30.000000000000114],[500.00000000000006,30.000000000000114],[500.00000000000006,-219.99999999999983],[0,-219.99999999999983],[65.7419999999999,-200.62299999999988],[115.12700000000001,-170.5639999999999],[155.73799999999994,-114.981],[160,-49.999999999999886],[102.24599999999998,-92.57699999999966],[50.714999999999975,-109.7529999999997],[0,-119.99999999999983],[-75.33200000000002,-114.02399999999977],[-122.66100000000006,-86.34299999999996],[-160.00000000000009,-49.999999999999886],[-149.472,-123.67499999999984],[-104.565,-175.67199999999997],[-55.180000000000064,-210.02699999999976],[0,-219.99999999999983],[-500.00000000000017,-219.99999999999983],[-500.00000000000017,-469.9999999999998],[-200.00000000000003,-469.9999999999998],[-135.76700000000002,-429.66999999999996],[-80.00000000000003,-371.92999999999995],[-103.83200000000002,-307.98099999999994],[-174.87200000000004,-323.4769999999999],[-200.00000000000003,-370],[-249.66000000000003,-322.846],[-318.55100000000004,-310.429],[-320.00000000000006,-372.696],[-275.001,-430.90199999999993],[-200.00000000000003,-470],[200.00000000000006,-470],[264.233,-429.66999999999996],[319.99999999999994,-371.92999999999984],[296.16799999999995,-307.9809999999998],[225.128,-323.4769999999998],[199.99999999999994,-370],[150.33999999999997,-322.846],[81.44899999999996,-310.429],[79.99999999999994,-372.696],[124.99900000000002,-430.9019999999997],[199.99999999999994,-470],[500.00000000000006,-470],[500.00000000000006,-470],[500.00000000000006,-219.99999999999994],[0,-219.99999999999994],[0,-319.99999999999994],[0,-419.99999999999994],[0,-520],[0,-599.9999999999999]]</x:v>
+        <x:v>[[0,530.0000000000001],[500,530.0000000000001],[532.135,552.6470000000003],[560,590.0000000000001],[535.212,631.0790000000001],[500,650.0000000000001],[456.784,632.1230000000002],[440,590.0000000000001],[455.584,557.3260000000004],[500,530.0000000000001],[700,530.0000000000001],[734.08,552.919],[760,590.0000000000001],[736.108,632.245],[700,650.0000000000001],[661.26,634.7360000000002],[640,590.0000000000001],[652.609,552.8000000000001],[700,530.0000000000001],[1100,530.0000000000001],[1100,280.0000000000001],[600,280.0000000000001],[665.742,299.37700000000007],[715.127,329.43600000000004],[755.738,385.0190000000001],[760,450.0000000000001],[702.246,407.4230000000001],[650.715,390.24700000000007],[600,380],[524.668,385.9760000000001],[477.339,413.65700000000015],[440,450.0000000000001],[450.528,376.32500000000005],[495.435,324.3280000000001],[544.82,289.97300000000007],[600,280.0000000000001],[100,280.0000000000001],[100,30.000000000000114],[500,30.000000000000114],[532.135,52.647000000000276],[560,90.00000000000011],[535.212,131.07900000000006],[500,150.0000000000001],[456.784,132.12299999999993],[440,90.00000000000011],[455.584,57.326000000000136],[500,30.000000000000114],[700,30.000000000000114],[734.08,52.919000000000096],[760,90.00000000000011],[736.108,132.24500000000012],[700,150.0000000000001],[661.26,134.7360000000001],[640,90.00000000000011],[652.609,52.800000000000296],[700,30.000000000000114],[1100,30.000000000000114],[1100,-219.99999999999983],[600,-219.99999999999983],[665.742,-200.62299999999988],[715.127,-170.5639999999999],[755.738,-114.981],[760,-49.999999999999886],[702.246,-92.57699999999966],[650.715,-109.7529999999997],[600,-119.99999999999983],[524.668,-114.02399999999977],[477.339,-86.34299999999996],[440,-49.999999999999886],[450.528,-123.67499999999984],[495.435,-175.67199999999997],[544.82,-210.02699999999976],[600,-219.99999999999983],[100,-219.99999999999983],[100,-469.9999999999998],[400,-469.9999999999998],[464.233,-429.66999999999996],[520,-371.92999999999995],[496.168,-307.98099999999994],[425.128,-323.4769999999999],[400,-370],[350.34,-322.846],[281.449,-310.429],[280,-372.696],[324.999,-430.90199999999993],[400,-470],[800,-470],[864.233,-429.66999999999996],[920,-371.92999999999984],[896.168,-307.9809999999998],[825.128,-323.4769999999998],[800,-370],[750.34,-322.846],[681.449,-310.429],[680,-372.696],[724.999,-430.9019999999997],[800,-470],[1100,-470],[1100,-470],[1100,-219.99999999999994],[600,-219.99999999999994],[600,-319.99999999999994],[600,-419.99999999999994],[600,-520],[600,-599.9999999999999]]</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -522,7 +522,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>[[-500,380],[-318,380],[-321.079,462.949],[-281.365,543.012],[-222.487,606.915],[-155.945,644.823],[-89.402,621.413],[-26.692,594.171],[0,540],[26.692000000000007,594.1710000000002],[89.40199999999999,621.4130000000004],[155.94500000000005,644.8230000000002],[222.48700000000002,606.9150000000003],[281.36499999999995,543.0119999999998],[321.079,462.9490000000002],[318,380],[293.204,318.15099999999995],[241.44099999999997,261.5120000000003],[188.16699999999997,204.7750000000002],[120.77099999999996,164],[56.58600000000001,128.187],[0,100.00000000000023],[-56.58600000000001,128.187],[-120.77099999999996,164],[-188.167,204.77500000000032],[-241.44100000000003,261.5120000000003],[-293.204,318.15099999999995],[-318,380],[-130.318,380],[-72.981,447.485],[9.6,218.69],[93.469,522.538],[153.16,380],[318,380],[500,380],[500,-300],[318.00000000000017,-300],[321.079,-217.05099999999976],[281.36499999999995,-136.98800000000017],[222.48700000000002,-73.08499999999992],[155.94500000000005,-35.17699999999979],[89.40199999999999,-58.586999999999875],[26.692000000000007,-85.82899999999978],[0,-140.0000000000001],[-26.692000000000064,-85.82899999999978],[-89.40199999999999,-58.58699999999942],[-155.94500000000008,-35.17699999999979],[-222.48700000000002,-73.08499999999941],[-281.36499999999995,-136.98800000000017],[-321.079,-217.05099999999976],[-318.0000000000001,-300],[-293.204,-361.84900000000005],[-241.44100000000003,-418.4879999999997],[-188.167,-475.2249999999997],[-120.77099999999996,-516],[-56.58600000000001,-551.813],[0,-579.9999999999997],[56.58600000000001,-551.813],[120.77099999999996,-516],[188.1670000000001,-475.2249999999997],[241.44099999999997,-418.4879999999997],[293.204,-361.84900000000005],[318.00000000000017,-300],[130.31799999999998,-300],[72.98099999999994,-232.51499999999976],[-9.599999999999966,-461.30999999999995],[-93.469,-157.46199999999988],[-153.16,-300],[-318.0000000000001,-300],[-500,-300],[-500,0],[-408.478,70.393],[-322.612,104.022],[-248.058,83.92],[-176.332,69.473],[-110.262,43.715],[-55.503,20.784]]</x:v>
+        <x:v>[[0,380],[182,380],[178.921,462.949],[218.635,543.012],[277.513,606.915],[344.055,644.823],[410.598,621.413],[473.308,594.171],[500,540],[526.692,594.1710000000002],[589.402,621.4130000000004],[655.945,644.8230000000002],[722.487,606.9150000000003],[781.365,543.0119999999998],[821.079,462.9490000000002],[818,380],[793.204,318.15099999999995],[741.441,261.5120000000003],[688.167,204.7750000000002],[620.771,164],[556.586,128.187],[500,100.00000000000023],[443.414,128.187],[379.229,164],[311.833,204.77500000000032],[258.559,261.5120000000003],[206.796,318.15099999999995],[182,380],[369.682,380],[427.019,447.485],[509.6,218.69],[593.469,522.538],[653.16,380],[818,380],[1000,380],[1000,-300],[818,-300],[821.079,-217.05099999999976],[781.365,-136.98800000000017],[722.487,-73.08499999999992],[655.945,-35.17699999999979],[589.402,-58.586999999999875],[526.692,-85.82899999999978],[500,-140.0000000000001],[473.308,-85.82899999999978],[410.598,-58.58699999999942],[344.055,-35.17699999999979],[277.513,-73.08499999999941],[218.635,-136.98800000000017],[178.921,-217.05099999999976],[182,-300],[206.796,-361.84900000000005],[258.559,-418.4879999999997],[311.833,-475.2249999999997],[379.229,-516],[443.414,-551.813],[500,-579.9999999999997],[556.586,-551.813],[620.771,-516],[688.167,-475.2249999999997],[741.441,-418.4879999999997],[793.204,-361.84900000000005],[818,-300],[630.318,-300],[572.981,-232.51499999999976],[490.4,-461.30999999999995],[406.531,-157.46199999999988],[346.84,-300],[182,-300],[0,-300],[0,0],[91.522,70.393],[177.388,104.022],[251.942,83.92],[323.668,69.473],[389.738,43.715],[444.497,20.784]]</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
@@ -533,7 +533,7 @@
         <x:v>[[2,2],[5,2],[8,2],[11,2],[14,2],[18,2],[21,2],[24,2],[27,2],[31,2],[35,2],[39,2],[43,2],[47,2],[50,2],[54,2],[58,2],[62,2],[66,2]]</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>[[-200,850],[-200,630],[-50,630],[-50,530],[-200,530],[-200,430],[-50,430],[50,430],[200,430],[200,530],[50,530],[50,630],[200,630],[450,630],[450,330],[340,330],[-340,330],[-170,160],[0,330],[170,160],[340,330],[340,160],[-340,160],[-170,-10],[0,160],[170,-10],[340,160],[340,-10],[-340,-10],[-170,-180],[0,-10],[170,-180],[340,-10],[340,-180],[-340,-180],[-170,-350],[0,-180],[170,-350],[340,-180],[340,-480],[170,-350],[0,-480],[-170,-350],[-340,-480],[-340,-350],[0,-350],[0,-400],[0,-450],[0,-500],[0,-550]]</x:v>
+        <x:v>[[0,850],[0,630],[150,630],[150,530],[0,530],[0,430],[150,430],[250,430],[400,430],[400,530],[250,530],[250,630],[400,630],[650,630],[650,330],[540,330],[-140,330],[30,160],[200,330],[370,160],[540,330],[540,160],[-140,160],[30,-10],[200,160],[370,-10],[540,160],[540,-10],[-140,-10],[30,-180],[200,-10],[370,-180],[540,-10],[540,-180],[-140,-180],[30,-350],[200,-180],[370,-350],[540,-180],[540,-480],[370,-350],[200,-480],[30,-350],[-140,-480],[-140,-350],[200,-350],[200,-400],[200,-450],[200,-500],[200,-550]]</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
@@ -550,7 +550,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra763d1ceb53448c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ee833f63073449a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -688,7 +688,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc93745219a5f4f8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f26cb625fa640e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>